<commit_message>
Implement paper TODOs, make the JEP version compliant, add a PNAS version
- TODOs: WVS and Gallup on equal footing; region R² in abstract and intro;
  six continents; bold cells (highest R² per row, shares > 0.5); CV R² of the
  best income measure; Gallup subsection; happiest country-years; shares of
  the R² gap in percent; Deaton (2008) growth test (no negative relation)
- JEP: appendix moved to a separate Online Appendix (not counted in the
  12,000-word limit; cross-references via xr-hyper); footnotes turned into
  text; data availability statement; counted manuscript about 9,500 words
- PNAS: wellbeing_pnas.tex (abstract, significance statement, Results,
  Discussion, Materials and Methods, 4 display items, numbered references)
  and SI Appendix wellbeing_pnas_si.tex

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Le5VwdePcLrubzQ7GsXPNq
</commit_message>
<xml_diff>
--- a/tables/main/r2_income_all_regions.xlsx
+++ b/tables/main/r2_income_all_regions.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Region: World Bank (7)</t>
   </si>
   <si>
-    <t xml:space="preserve">Region: continents (5)</t>
+    <t xml:space="preserve">Region: continents (6)</t>
   </si>
   <si>
     <t xml:space="preserve">Happy</t>
@@ -488,7 +488,7 @@
         <v>0.111010906564617</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0819477344673852</v>
+        <v>0.0920894413401486</v>
       </c>
     </row>
     <row r="3">
@@ -529,7 +529,7 @@
         <v>0.23217511345087</v>
       </c>
       <c r="M3" t="n">
-        <v>0.233360482813203</v>
+        <v>0.234128959896389</v>
       </c>
     </row>
     <row r="4">
@@ -570,7 +570,7 @@
         <v>0.15755178520278</v>
       </c>
       <c r="M4" t="n">
-        <v>0.098293512189043</v>
+        <v>0.0991330101013062</v>
       </c>
     </row>
     <row r="5">
@@ -611,7 +611,7 @@
         <v>0.225101193368732</v>
       </c>
       <c r="M5" t="n">
-        <v>0.217134085878367</v>
+        <v>0.217500332030212</v>
       </c>
     </row>
     <row r="6">
@@ -652,7 +652,7 @@
         <v>0.154281023410774</v>
       </c>
       <c r="M6" t="n">
-        <v>0.154501749335799</v>
+        <v>0.155662793827058</v>
       </c>
     </row>
     <row r="7">
@@ -693,7 +693,7 @@
         <v>0.229869568355362</v>
       </c>
       <c r="M7" t="n">
-        <v>0.234790186077392</v>
+        <v>0.234855641380854</v>
       </c>
     </row>
     <row r="8">
@@ -734,7 +734,7 @@
         <v>0.204786227406024</v>
       </c>
       <c r="M8" t="n">
-        <v>0.185292541167775</v>
+        <v>0.186586790162678</v>
       </c>
     </row>
     <row r="9">
@@ -775,7 +775,7 @@
         <v>0.1714646123365</v>
       </c>
       <c r="M9" t="n">
-        <v>0.135537814382107</v>
+        <v>0.140110880071311</v>
       </c>
     </row>
     <row r="10">
@@ -816,7 +816,7 @@
         <v>0.185780053761957</v>
       </c>
       <c r="M10" t="n">
-        <v>0.167607263288884</v>
+        <v>0.170008481101245</v>
       </c>
     </row>
     <row r="11">
@@ -857,7 +857,7 @@
         <v>0.23217511345087</v>
       </c>
       <c r="M11" t="n">
-        <v>0.234790186077392</v>
+        <v>0.234855641380854</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement paper TODOs, verify the bibliography, add cover letters and reviews
- Appendix back in wellbeing.tex; continents redefined (three definitions
  compared); median income (PIP) and household consumption in the correlates;
  country-clustered bootstrap CIs for the main R² and LMG shares; replication
  of Deaton (2008) on growth; shares in percent; wording edits; new references
- Bibliography checked against Crossref/DataCite, DOIs and URLs added
- ORCID; PNAS: direct submission, title kept
- Cover letters (PNAS, JEP) as .docx; referee-style reviews for both

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Le5VwdePcLrubzQ7GsXPNq
</commit_message>
<xml_diff>
--- a/tables/main/r2_income_all_regions.xlsx
+++ b/tables/main/r2_income_all_regions.xlsx
@@ -488,7 +488,7 @@
         <v>0.111010906564617</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0920894413401486</v>
+        <v>0.0898082386875273</v>
       </c>
     </row>
     <row r="3">
@@ -529,7 +529,7 @@
         <v>0.23217511345087</v>
       </c>
       <c r="M3" t="n">
-        <v>0.234128959896389</v>
+        <v>0.24774773010099</v>
       </c>
     </row>
     <row r="4">
@@ -570,7 +570,7 @@
         <v>0.15755178520278</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0991330101013062</v>
+        <v>0.0984902985117729</v>
       </c>
     </row>
     <row r="5">
@@ -611,7 +611,7 @@
         <v>0.225101193368732</v>
       </c>
       <c r="M5" t="n">
-        <v>0.217500332030212</v>
+        <v>0.229562580291188</v>
       </c>
     </row>
     <row r="6">
@@ -652,7 +652,7 @@
         <v>0.154281023410774</v>
       </c>
       <c r="M6" t="n">
-        <v>0.155662793827058</v>
+        <v>0.166680433222706</v>
       </c>
     </row>
     <row r="7">
@@ -693,7 +693,7 @@
         <v>0.229869568355362</v>
       </c>
       <c r="M7" t="n">
-        <v>0.234855641380854</v>
+        <v>0.237243716184806</v>
       </c>
     </row>
     <row r="8">
@@ -734,7 +734,7 @@
         <v>0.204786227406024</v>
       </c>
       <c r="M8" t="n">
-        <v>0.186586790162678</v>
+        <v>0.186786758590563</v>
       </c>
     </row>
     <row r="9">
@@ -775,7 +775,7 @@
         <v>0.1714646123365</v>
       </c>
       <c r="M9" t="n">
-        <v>0.140110880071311</v>
+        <v>0.139736629094961</v>
       </c>
     </row>
     <row r="10">
@@ -816,7 +816,7 @@
         <v>0.185780053761957</v>
       </c>
       <c r="M10" t="n">
-        <v>0.170008481101245</v>
+        <v>0.174507048085564</v>
       </c>
     </row>
     <row r="11">
@@ -857,7 +857,7 @@
         <v>0.23217511345087</v>
       </c>
       <c r="M11" t="n">
-        <v>0.234855641380854</v>
+        <v>0.24774773010099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>